<commit_message>
feat(phase-55): enterprise cloud foundation, gemini adapter, durable memory, and jwt auth
</commit_message>
<xml_diff>
--- a/AI_Operating_Platform_Roadmap.xlsx
+++ b/AI_Operating_Platform_Roadmap.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -611,9 +611,9 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>[AOP-MODEL-GEMINI]
-Adaptador de Modelo Google Gemini / Vertex AI
-Área: Models (v1.2)</t>
+          <t>[AOP-V1-EXIT]
+Certificación Final de Criterios de Producción
+Área: Governance (v1.2)</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr"/>
@@ -631,13 +631,7 @@
       <c r="H5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>[AOP-AUTH]
-Proveedor de Autenticación OIDC / JWT Producción
-Área: Security (v1.2)</t>
-        </is>
-      </c>
+      <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr"/>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr"/>
@@ -653,13 +647,7 @@
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>[AOP-NETWORK]
-Topología de Red y Proxy Reverso de Producción
-Área: Security (v1.2)</t>
-        </is>
-      </c>
+      <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr"/>
       <c r="C7" s="5" t="inlineStr"/>
       <c r="D7" s="5" t="inlineStr"/>
@@ -675,13 +663,7 @@
       <c r="H7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>[AOP-MEMORY]
-Pasarela de Memoria Duradera SQLite
-Área: Memory (v1.2)</t>
-        </is>
-      </c>
+      <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr"/>
       <c r="C8" s="5" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr"/>
@@ -697,13 +679,7 @@
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>[AOP-API-SURFACES]
-Política de Convergencia de Rutas /api/v1
-Área: Platform API (v1.2)</t>
-        </is>
-      </c>
+      <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr"/>
       <c r="C9" s="5" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr"/>
@@ -719,13 +695,7 @@
       <c r="H9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>[AOP-V1-EXIT]
-Certificación Final de Criterios de Producción
-Área: Governance (v1.2)</t>
-        </is>
-      </c>
+      <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr"/>
       <c r="C10" s="5" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr"/>
@@ -1043,6 +1013,86 @@
       </c>
       <c r="G29" s="5" t="inlineStr"/>
       <c r="H29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-MODEL-GEMINI]
+Adaptador de Modelo Google Gemini / Vertex AI
+Área: Models (v1.2)</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="5" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-AUTH]
+Proveedor de Autenticación OIDC / JWT Producción
+Área: Security (v1.2)</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr"/>
+      <c r="H31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr"/>
+      <c r="B32" s="5" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-NETWORK]
+Topología de Red y Proxy Reverso de Producción
+Área: Security (v1.2)</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-MEMORY]
+Pasarela de Memoria Duradera SQLite
+Área: Memory (v1.2)</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-API-SURFACES]
+Política de Convergencia de Rutas /api/v1
+Área: Platform API (v1.2)</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1202,7 +1252,7 @@
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1263,7 +1313,7 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Resuelta</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -1273,17 +1323,17 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Peticiones a modelos Google desviadas a Stub</t>
+          <t>Resuelta en Prompt 101 / Fase 55 con GeminiModelGateway</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Implementar GeminiModelGateway en src/infrastructure/model/gemini/</t>
+          <t>Implementado GeminiModelGateway en src/infrastructure/model/gemini/</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>v1.2 (AOP-MODEL-GEMINI)</t>
+          <t>v1.2 (AOP-MODEL-GEMINI) - CERRADA</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1350,7 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Resuelta</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -1310,17 +1360,17 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Pérdida de contexto de agente si el proceso se reinicia</t>
+          <t>Resuelta en Prompt 101 / Fase 55 con SqliteMemoryGateway</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Implementar SqliteMemoryGateway relacional duradero</t>
+          <t>Implementado SqliteMemoryGateway relacional duradero</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>v1.2 (AOP-MEMORY)</t>
+          <t>v1.2 (AOP-MEMORY) - CERRADA</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1387,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Resuelta</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -1347,17 +1397,17 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Apto para entornos locales; insuficiente para internet público abierto</t>
+          <t>Resuelta en Prompt 101 / Fase 55 con JwtTokenVerifier</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Integrar proveedor formal JWT con rotación asimétrica</t>
+          <t>Integrado JwtTokenVerifier asimétrico RS256/ES256</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>v1.2 (AOP-AUTH)</t>
+          <t>v1.2 (AOP-AUTH) - CERRADA</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1424,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Resuelta</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -1384,7 +1434,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>No exponer directamente a 0.0.0.0 sin capa perimetral HTTPS</t>
+          <t>Resuelta en Prompt 101 / Fase 55 con Caddy/Nginx manifests</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -1394,7 +1444,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>v1.2 (AOP-NETWORK)</t>
+          <t>v1.2 (AOP-NETWORK) - CERRADA</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1461,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Resuelta</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -1421,7 +1471,7 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Riesgo de confusión en desarrolladores externos</t>
+          <t>Resuelta en Prompt 101 / Fase 55 con cabeceras RFC 8594</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
@@ -1431,7 +1481,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>v1.2 (AOP-API-SURFACES)</t>
+          <t>v1.2 (AOP-API-SURFACES) - CERRADA</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2435,6 +2485,134 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>ADR 0023</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Google Gemini Model Gateway Adapter</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>0023-google-gemini-model-gateway.md</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Adaptador oficial para Google Gemini y Vertex AI con streaming y JSON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>ADR 0024</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>SQLite Durable Memory Gateway</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>0024-sqlite-durable-memory-gateway.md</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Persistencia relacional duradera para memoria indexada por agente y sesión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>ADR 0025</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Asymmetric JWT &amp; Key Rotation</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>0025-asymmetric-jwt-and-key-rotation.md</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Verificación criptográfica RS256/ES256 y rotación dinámica de claves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>ADR 0026</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Production Reverse Proxy &amp; TLS</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>0026-production-reverse-proxy-and-tls.md</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Manifiestos Nginx/Caddy con terminación TLS y rate limiting perimetral.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2446,7 +2624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2454,7 +2632,7 @@
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
@@ -2462,7 +2640,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MATRIZ DE TRAZABILIDAD DE PROMPTS (PROMPTS 94 AL 100)</t>
+          <t>MATRIZ DE TRAZABILIDAD DE PROMPTS (PROMPTS 94 AL 101)</t>
         </is>
       </c>
     </row>
@@ -2798,6 +2976,48 @@
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 101</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Phase 55</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Enterprise Cloud Foundation &amp; Real Model Expansion</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Gemini Gateway, SqliteMemoryGateway, JWT RS256/ES256, Caddy/Nginx TLS, RFC 8594</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>src/infrastructure/, deploy/</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>19 tests pass (985 total)</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>feat(phase-55)</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2819,7 +3039,7 @@
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2879,7 +3099,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>966 PASS (0 FAIL)</t>
+          <t>985 PASS (0 FAIL)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -2930,7 +3150,7 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>25 Iniciativas (80.6%)</t>
+          <t>30 Iniciativas (96.8%)</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -2947,12 +3167,12 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>6 Iniciativas (19.4%)</t>
+          <t>1 Iniciativa (3.2%)</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Programadas para versión v1.2.0</t>
+          <t>AOP-V1-EXIT (Certificación de salida)</t>
         </is>
       </c>
     </row>
@@ -3015,12 +3235,12 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>32 ADRs Catalogados</t>
+          <t>36 ADRs Catalogados</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>docs/decisions/ (ADR 0001 al 0022 + Serie ADR)</t>
+          <t>docs/decisions/ (ADR 0001 al 0026 + Serie ADR-001..010)</t>
         </is>
       </c>
     </row>
@@ -3126,14 +3346,14 @@
         <v>6</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>OPERACIONAL (Memoria en backlog)</t>
+          <t>MADURA (SQLite WAL + Memoria Duradera)</t>
         </is>
       </c>
     </row>
@@ -3144,17 +3364,17 @@
         </is>
       </c>
       <c r="B24" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>OPERACIONAL (Convergencia en backlog)</t>
+          <t>OPERACIONAL (Convergencia RFC 8594)</t>
         </is>
       </c>
     </row>
@@ -3165,17 +3385,17 @@
         </is>
       </c>
       <c r="B25" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>OPERACIONAL (Gemini en backlog)</t>
+          <t>OPERACIONAL (OpenAI, Anthropic, Ollama, Gemini)</t>
         </is>
       </c>
     </row>
@@ -3186,17 +3406,17 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C26" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>OPERACIONAL (Support Agent en backlog)</t>
+          <t>OPERACIONAL (Tentaciones + Vehicle Parts)</t>
         </is>
       </c>
     </row>
@@ -3228,17 +3448,17 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C28" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>OPERACIONAL (OIDC / TLS en backlog)</t>
+          <t>OPERACIONAL (Auth JWT + TLS listos; V1-Exit backlog)</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3485,7 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
@@ -5311,9 +5531,9 @@
           <t>Gateway oficial para Google Gemini 1.5/2.0 Pro/Flash vía API REST de Google Cloud.</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
-        <is>
-          <t>BACKLOG</t>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -5333,37 +5553,37 @@
       </c>
       <c r="I30" s="9" t="inlineStr">
         <is>
+          <t>src/infrastructure/model/gemini/</t>
+        </is>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>8 tests</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0023-google-gemini-model-gateway.md</t>
+        </is>
+      </c>
+      <c r="L30" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 101</t>
+        </is>
+      </c>
+      <c r="M30" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N30" s="9" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J30" s="9" t="inlineStr">
-        <is>
-          <t>0 tests</t>
-        </is>
-      </c>
-      <c r="K30" s="9" t="inlineStr">
-        <is>
-          <t>docs/TECHNICAL_DEBT.md</t>
-        </is>
-      </c>
-      <c r="L30" s="9" t="inlineStr">
-        <is>
-          <t>Prompt 101+</t>
-        </is>
-      </c>
-      <c r="M30" s="9" t="inlineStr">
-        <is>
-          <t>Platform Core</t>
-        </is>
-      </c>
-      <c r="N30" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="O30" s="9" t="inlineStr">
         <is>
-          <t>GAP-01</t>
+          <t>GAP-01 Resuelto</t>
         </is>
       </c>
     </row>
@@ -5385,12 +5605,12 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Servicio formal de validación JWT con rotación asimétrica de claves y gestión de roles RBAC.</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>BACKLOG</t>
+          <t>Servicio formal de validación JWT con rotación asimétrica de claves (RS256/ES256) y gestión de roles.</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="F31" s="11" t="inlineStr">
@@ -5410,37 +5630,37 @@
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
+          <t>src/infrastructure/security/jwt-token-verifier.ts</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>4 tests</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0025-asymmetric-jwt-and-key-rotation.md</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 101</t>
+        </is>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N31" s="9" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J31" s="9" t="inlineStr">
-        <is>
-          <t>0 tests</t>
-        </is>
-      </c>
-      <c r="K31" s="9" t="inlineStr">
-        <is>
-          <t>docs/TECHNICAL_DEBT.md</t>
-        </is>
-      </c>
-      <c r="L31" s="9" t="inlineStr">
-        <is>
-          <t>Prompt 101+</t>
-        </is>
-      </c>
-      <c r="M31" s="9" t="inlineStr">
-        <is>
-          <t>Platform Core</t>
-        </is>
-      </c>
-      <c r="N31" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="O31" s="9" t="inlineStr">
         <is>
-          <t>GAP-03</t>
+          <t>GAP-03 Resuelto</t>
         </is>
       </c>
     </row>
@@ -5462,12 +5682,12 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Configuración declarativa de Nginx/Caddy con terminación TLS, rate limiting perimetral y CORS restrictivo.</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>BACKLOG</t>
+          <t>Configuración declarativa de Nginx/Caddy con terminación TLS, rate limiting perimetral y Docker Compose.</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
@@ -5487,37 +5707,37 @@
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
+          <t>deploy/</t>
+        </is>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>Manifests</t>
+        </is>
+      </c>
+      <c r="K32" s="9" t="inlineStr">
+        <is>
+          <t>docs/PRODUCTION_NETWORK_TOPOLOGY.md</t>
+        </is>
+      </c>
+      <c r="L32" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 101</t>
+        </is>
+      </c>
+      <c r="M32" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N32" s="9" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J32" s="9" t="inlineStr">
-        <is>
-          <t>0 tests</t>
-        </is>
-      </c>
-      <c r="K32" s="9" t="inlineStr">
-        <is>
-          <t>docs/TECHNICAL_DEBT.md</t>
-        </is>
-      </c>
-      <c r="L32" s="9" t="inlineStr">
-        <is>
-          <t>Prompt 101+</t>
-        </is>
-      </c>
-      <c r="M32" s="9" t="inlineStr">
-        <is>
-          <t>Platform Core</t>
-        </is>
-      </c>
-      <c r="N32" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="O32" s="9" t="inlineStr">
         <is>
-          <t>GAP-04</t>
+          <t>GAP-04 Resuelto</t>
         </is>
       </c>
     </row>
@@ -5542,9 +5762,9 @@
           <t>Adaptador SqliteMemoryGateway con persistencia relacional indexada por ámbito de agente y sesión.</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>BACKLOG</t>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
@@ -5564,37 +5784,37 @@
       </c>
       <c r="I33" s="9" t="inlineStr">
         <is>
+          <t>src/infrastructure/memory/sqlite-memory-gateway.ts</t>
+        </is>
+      </c>
+      <c r="J33" s="9" t="inlineStr">
+        <is>
+          <t>6 tests</t>
+        </is>
+      </c>
+      <c r="K33" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0024-sqlite-durable-memory-gateway.md</t>
+        </is>
+      </c>
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 101</t>
+        </is>
+      </c>
+      <c r="M33" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N33" s="9" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J33" s="9" t="inlineStr">
-        <is>
-          <t>0 tests</t>
-        </is>
-      </c>
-      <c r="K33" s="9" t="inlineStr">
-        <is>
-          <t>docs/TECHNICAL_DEBT.md</t>
-        </is>
-      </c>
-      <c r="L33" s="9" t="inlineStr">
-        <is>
-          <t>Prompt 101+</t>
-        </is>
-      </c>
-      <c r="M33" s="9" t="inlineStr">
-        <is>
-          <t>Platform Core</t>
-        </is>
-      </c>
-      <c r="N33" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="O33" s="9" t="inlineStr">
         <is>
-          <t>GAP-02</t>
+          <t>GAP-02 Resuelto</t>
         </is>
       </c>
     </row>
@@ -5616,12 +5836,12 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Eliminación planificada del alias /api/platform/v1 en favor de /api/v1 con avisos de deprecación.</t>
-        </is>
-      </c>
-      <c r="E34" s="12" t="inlineStr">
-        <is>
-          <t>BACKLOG</t>
+          <t>Eliminación planificada del alias /api/platform/v1 en favor de /api/v1 con avisos RFC 8594.</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
@@ -5641,37 +5861,37 @@
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
+          <t>src/platform/api/http-router.ts</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>1 test</t>
+        </is>
+      </c>
+      <c r="K34" s="9" t="inlineStr">
+        <is>
+          <t>docs/TECHNICAL_DEBT.md</t>
+        </is>
+      </c>
+      <c r="L34" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 101</t>
+        </is>
+      </c>
+      <c r="M34" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N34" s="9" t="inlineStr">
+        <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J34" s="9" t="inlineStr">
-        <is>
-          <t>0 tests</t>
-        </is>
-      </c>
-      <c r="K34" s="9" t="inlineStr">
-        <is>
-          <t>docs/TECHNICAL_DEBT.md</t>
-        </is>
-      </c>
-      <c r="L34" s="9" t="inlineStr">
-        <is>
-          <t>Prompt 101+</t>
-        </is>
-      </c>
-      <c r="M34" s="9" t="inlineStr">
-        <is>
-          <t>Platform Core</t>
-        </is>
-      </c>
-      <c r="N34" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="O34" s="9" t="inlineStr">
         <is>
-          <t>GAP-05</t>
+          <t>GAP-05 Resuelto</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -6291,7 +6511,7 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Línea Base Canónica Actual</t>
+          <t>Línea Base Fase 54</t>
         </is>
       </c>
     </row>
@@ -6303,25 +6523,57 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Gateway Gemini, OIDC/JWT, proxy reverso TLS</t>
+          <t>Gateway Gemini, OIDC/JWT, proxy reverso TLS, memoria SQLite</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Certificación formal para nube pública</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
+          <t>985 tests PASS, 11 suites, 0 runtime deps</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>985 tests PASS</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Línea Base Canónica Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>v1.2.1 Production Certification</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Certificación formal de producción y pruebas de carga</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Criterios de salida formal v1.0/v1.2 completados</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>0 tests (Backlog)</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>Próxima fase</t>
         </is>
@@ -6338,7 +6590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -6901,6 +7153,70 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>AOP-MEMORY</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Memoria Duradera SQLite</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>AOP-PERS-001</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Motor SQLite Nativo</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Persistencia Relacional</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>AOP-API-SURFACES</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Convergencia de Rutas</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>AOP-PROD-001</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Servidor HTTP Nativo</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Deprecación RFC 8594</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6912,7 +7228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -7360,7 +7676,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Model Gateways</t>
+          <t>SqliteMemoryGateway</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -7370,32 +7686,32 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Adaptadores para OpenAI, Anthropic, Ollama y Stub</t>
+          <t>Persistencia relacional duradera de memoria de agentes</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>node:http, node:https</t>
+          <t>node:sqlite nativo</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>ModelGateway.execute()</t>
+          <t>MemoryGateway</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Ocultación de API keys en logs</t>
+          <t>SQL parametrizado, índice scope/key</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Ninguna</t>
+          <t>data/app.db (platform_memory)</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>model.requested/completed</t>
+          <t>Métricas de operaciones</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
@@ -7407,45 +7723,186 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>Model Gateways</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Adaptadores para OpenAI, Anthropic, Ollama, Gemini y Stub</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>node:http, node:https</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>ModelGateway.execute()</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Ocultación de API keys en logs</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>model.requested/completed</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED / OPERATIONAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>JwtTokenVerifier</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Validación criptográfica JWT asimétrica (RS256/ES256)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>node:crypto nativo</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>TokenVerifier</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Rotación dinámica y revocación kid</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Auditoría de autenticación</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED / OPERATIONAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Reverse Proxy Topology</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Terminación TLS, rate limiting y CORS perimetral</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Nginx / Caddy v2</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>https://localhost:443/</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Terminación TLS + Headers HSTS/CSP</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Ninguna</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Access logs y métricas</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>CONFIGURED / DEPLOYABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>BrotherPrinterAdapter</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Control y spooler de impresora comercial USB</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>APIs nativas de SO</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>BusinessDeviceAdapter</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Validación MIME y límites de cola</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>Cola en memoria</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>Métricas de trabajos</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>IMPLEMENTED (Hardware Offline)</t>
         </is>
@@ -7683,11 +8140,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
@@ -8105,6 +8562,80 @@
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>SEC-011</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Autenticación Asimétrica JWT (RS256/ES256)</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>jwt-token-verifier.ts</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>4 tests pass</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0025-asymmetric-jwt-and-key-rotation.md</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>SEC-012</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Terminación TLS y Seguridad Perimetral</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>CONFIGURED</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>deploy/nginx/, deploy/caddy/</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Config checks pass</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>docs/PRODUCTION_NETWORK_TOPOLOGY.md</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
@@ -8135,7 +8666,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REGISTRO OFICIAL DE SUITES DE PRUEBAS (966 TESTS PASS)</t>
+          <t>REGISTRO OFICIAL DE SUITES DE PRUEBAS (985 TESTS PASS)</t>
         </is>
       </c>
     </row>
@@ -8208,18 +8739,18 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>sqlite-persistence.test.ts, sqlite-durable-events.test.ts</t>
+          <t>sqlite-persistence.test.ts, sqlite-memory-gateway.test.ts</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>node:sqlite nativo, transacciones atómicas, OCC y WAL</t>
+          <t>node:sqlite nativo, transacciones atómicas, memoria duradera y WAL</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
@@ -8264,18 +8795,18 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>model-gateway-contracts.test.ts, ollama-model-gateway.test.ts</t>
+          <t>model-gateway-contracts.test.ts, gemini-model-gateway.test.ts</t>
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Paridad de contratos para OpenAI, Anthropic, Ollama y Stub</t>
+          <t>Paridad de contratos para OpenAI, Anthropic, Ollama, Gemini y Stub</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -8348,18 +8879,18 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>security-boundaries.test.ts, authorization-rbac.test.ts</t>
+          <t>security-boundaries.test.ts, jwt-authentication.test.ts</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D10" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Gobernanza default-deny, límites multi-tenant y auditoría</t>
+          <t>Gobernanza default-deny, firmas asimétricas JWT y auditoría</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -8376,18 +8907,18 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>api.test.ts, diagnostics-api.test.ts, operations-api.test.ts</t>
+          <t>api.test.ts, diagnostics-api.test.ts, api-surface-deprecation.test.ts</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Rutas REST, rate limiting, esquemas DTO y trazas forenses</t>
+          <t>Rutas REST, convergencia RFC 8594, rate limiting y trazas</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -8464,7 +8995,7 @@
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>966</v>
+        <v>985</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat(phase-70): integrate autonomous operations governance and control plane
</commit_message>
<xml_diff>
--- a/AI_Operating_Platform_Roadmap.xlsx
+++ b/AI_Operating_Platform_Roadmap.xlsx
@@ -23,7 +23,7 @@
     <sheet name="14_DASHBOARD" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_MASTER_ROADMAP'!$A$4:$O$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_MASTER_ROADMAP'!$A$4:$O$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -103,14 +103,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -147,11 +147,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -159,16 +159,16 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -538,14 +538,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="49" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -609,17 +609,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>[AOP-V1-EXIT]
 Certificación Final de Criterios de Producción
-Área: Governance (v1.2)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
+Área: Governance (v1.3)</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
           <t>[AOP-CORE-001]
@@ -627,15 +627,15 @@
 Área: Core Engine (v0.1)</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
           <t>[AOP-CORE-002]
@@ -643,15 +643,15 @@
 Área: Core Engine (v0.2)</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
           <t>[AOP-CORE-003]
@@ -659,15 +659,15 @@
 Área: Tools (v0.3)</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr"/>
       <c r="F8" s="6" t="inlineStr">
         <is>
           <t>[AOP-CORE-004]
@@ -675,15 +675,15 @@
 Área: Orchestration (v0.4)</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr"/>
-      <c r="E9" s="5" t="inlineStr"/>
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr"/>
       <c r="F9" s="6" t="inlineStr">
         <is>
           <t>[AOP-CORE-005]
@@ -691,15 +691,15 @@
 Área: Memory (v0.5)</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr"/>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="6" t="inlineStr">
         <is>
           <t>[AOP-CORE-006]
@@ -707,15 +707,15 @@
 Área: Security (v0.6)</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr"/>
-      <c r="E11" s="5" t="inlineStr"/>
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
       <c r="F11" s="6" t="inlineStr">
         <is>
           <t>[AOP-CORE-007]
@@ -723,15 +723,15 @@
 Área: Agents (v0.8)</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr"/>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="5" t="inlineStr"/>
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="6" t="inlineStr">
         <is>
           <t>[AOP-CORE-008]
@@ -739,15 +739,15 @@
 Área: Autonomy (v0.9)</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr"/>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr"/>
-      <c r="E13" s="5" t="inlineStr"/>
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr"/>
       <c r="F13" s="6" t="inlineStr">
         <is>
           <t>[AOP-PERS-001]
@@ -755,15 +755,15 @@
 Área: Persistence (v0.10)</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr"/>
-      <c r="B14" s="5" t="inlineStr"/>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr"/>
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="6" t="inlineStr">
         <is>
           <t>[AOP-PERS-002]
@@ -771,15 +771,15 @@
 Área: Persistence (v0.10)</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr"/>
-      <c r="B15" s="5" t="inlineStr"/>
-      <c r="C15" s="5" t="inlineStr"/>
-      <c r="D15" s="5" t="inlineStr"/>
-      <c r="E15" s="5" t="inlineStr"/>
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
       <c r="F15" s="6" t="inlineStr">
         <is>
           <t>[AOP-PERS-003]
@@ -787,15 +787,15 @@
 Área: Persistence (v0.11)</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr"/>
-      <c r="B16" s="5" t="inlineStr"/>
-      <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="6" t="inlineStr">
         <is>
           <t>[AOP-PERS-004]
@@ -803,15 +803,15 @@
 Área: Persistence (v0.12)</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr"/>
-      <c r="H16" s="5" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr"/>
-      <c r="B17" s="5" t="inlineStr"/>
-      <c r="C17" s="5" t="inlineStr"/>
-      <c r="D17" s="5" t="inlineStr"/>
-      <c r="E17" s="5" t="inlineStr"/>
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr"/>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>[AOP-RECV-001]
@@ -819,15 +819,15 @@
 Área: Recovery (v0.13)</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr"/>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr"/>
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="6" t="inlineStr">
         <is>
           <t>[AOP-PERS-005]
@@ -835,15 +835,15 @@
 Área: Persistence (v0.13)</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
-      <c r="H18" s="5" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr"/>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr"/>
-      <c r="E19" s="5" t="inlineStr"/>
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="4" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr"/>
       <c r="F19" s="6" t="inlineStr">
         <is>
           <t>[AOP-PROD-001]
@@ -851,15 +851,15 @@
 Área: Platform API (v1.0)</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr"/>
+      <c r="H19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr"/>
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr"/>
       <c r="F20" s="6" t="inlineStr">
         <is>
           <t>[AOP-PROD-002]
@@ -867,15 +867,15 @@
 Área: Platform Client (v1.0)</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr"/>
-      <c r="B21" s="5" t="inlineStr"/>
-      <c r="C21" s="5" t="inlineStr"/>
-      <c r="D21" s="5" t="inlineStr"/>
-      <c r="E21" s="5" t="inlineStr"/>
+      <c r="A21" s="4" t="inlineStr"/>
+      <c r="B21" s="4" t="inlineStr"/>
+      <c r="C21" s="4" t="inlineStr"/>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr"/>
       <c r="F21" s="6" t="inlineStr">
         <is>
           <t>[AOP-PROD-003]
@@ -883,15 +883,15 @@
 Área: Web UI (v1.1)</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr"/>
-      <c r="B22" s="5" t="inlineStr"/>
-      <c r="C22" s="5" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="5" t="inlineStr"/>
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="4" t="inlineStr"/>
       <c r="F22" s="6" t="inlineStr">
         <is>
           <t>[AOP-PROD-004]
@@ -899,15 +899,15 @@
 Área: Developer Platform (v1.1)</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr"/>
+      <c r="H22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-      <c r="B23" s="5" t="inlineStr"/>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr"/>
+      <c r="A23" s="4" t="inlineStr"/>
+      <c r="B23" s="4" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr"/>
       <c r="F23" s="6" t="inlineStr">
         <is>
           <t>[AOP-MODL-001]
@@ -915,15 +915,15 @@
 Área: Models (v1.1)</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr"/>
-      <c r="C24" s="5" t="inlineStr"/>
-      <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="5" t="inlineStr"/>
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr"/>
       <c r="F24" s="6" t="inlineStr">
         <is>
           <t>[AOP-MODL-002]
@@ -931,15 +931,15 @@
 Área: Models (v1.1)</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr"/>
-      <c r="H24" s="5" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
-      <c r="B25" s="5" t="inlineStr"/>
-      <c r="C25" s="5" t="inlineStr"/>
-      <c r="D25" s="5" t="inlineStr"/>
-      <c r="E25" s="5" t="inlineStr"/>
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="4" t="inlineStr"/>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr"/>
       <c r="F25" s="6" t="inlineStr">
         <is>
           <t>[AOP-MODL-003]
@@ -947,15 +947,15 @@
 Área: Models (v1.1)</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr"/>
-      <c r="H25" s="5" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="5" t="inlineStr"/>
-      <c r="C26" s="5" t="inlineStr"/>
-      <c r="D26" s="5" t="inlineStr"/>
-      <c r="E26" s="5" t="inlineStr"/>
+      <c r="A26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr"/>
       <c r="F26" s="6" t="inlineStr">
         <is>
           <t>[AOP-MODL-004]
@@ -963,15 +963,15 @@
 Área: Models (v1.1)</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr"/>
-      <c r="B27" s="5" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr"/>
-      <c r="D27" s="5" t="inlineStr"/>
-      <c r="E27" s="5" t="inlineStr"/>
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="4" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
       <c r="F27" s="6" t="inlineStr">
         <is>
           <t>[AOP-APP-001]
@@ -979,15 +979,15 @@
 Área: Applications (v1.0)</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr"/>
-      <c r="B28" s="5" t="inlineStr"/>
-      <c r="C28" s="5" t="inlineStr"/>
-      <c r="D28" s="5" t="inlineStr"/>
-      <c r="E28" s="5" t="inlineStr"/>
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="4" t="inlineStr"/>
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr"/>
       <c r="F28" s="6" t="inlineStr">
         <is>
           <t>[AOP-APP-002]
@@ -995,15 +995,15 @@
 Área: Applications (v1.1)</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr"/>
-      <c r="H28" s="5" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="5" t="inlineStr"/>
-      <c r="C29" s="5" t="inlineStr"/>
-      <c r="D29" s="5" t="inlineStr"/>
-      <c r="E29" s="5" t="inlineStr"/>
+      <c r="A29" s="4" t="inlineStr"/>
+      <c r="B29" s="4" t="inlineStr"/>
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr"/>
       <c r="F29" s="6" t="inlineStr">
         <is>
           <t>[AOP-DEV-001]
@@ -1011,15 +1011,15 @@
 Área: Devices (v1.1)</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr"/>
-      <c r="H29" s="5" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr"/>
-      <c r="B30" s="5" t="inlineStr"/>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="5" t="inlineStr"/>
-      <c r="E30" s="5" t="inlineStr"/>
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr"/>
       <c r="F30" s="6" t="inlineStr">
         <is>
           <t>[AOP-MODEL-GEMINI]
@@ -1027,15 +1027,15 @@
 Área: Models (v1.2)</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr"/>
-      <c r="H30" s="5" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr"/>
-      <c r="B31" s="5" t="inlineStr"/>
-      <c r="C31" s="5" t="inlineStr"/>
-      <c r="D31" s="5" t="inlineStr"/>
-      <c r="E31" s="5" t="inlineStr"/>
+      <c r="A31" s="4" t="inlineStr"/>
+      <c r="B31" s="4" t="inlineStr"/>
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
           <t>[AOP-AUTH]
@@ -1043,15 +1043,15 @@
 Área: Security (v1.2)</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr"/>
-      <c r="H31" s="5" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr"/>
-      <c r="B32" s="5" t="inlineStr"/>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr"/>
-      <c r="E32" s="5" t="inlineStr"/>
+      <c r="A32" s="4" t="inlineStr"/>
+      <c r="B32" s="4" t="inlineStr"/>
+      <c r="C32" s="4" t="inlineStr"/>
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="inlineStr"/>
       <c r="F32" s="6" t="inlineStr">
         <is>
           <t>[AOP-NETWORK]
@@ -1059,15 +1059,15 @@
 Área: Security (v1.2)</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr"/>
-      <c r="H32" s="5" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr"/>
-      <c r="B33" s="5" t="inlineStr"/>
-      <c r="C33" s="5" t="inlineStr"/>
-      <c r="D33" s="5" t="inlineStr"/>
-      <c r="E33" s="5" t="inlineStr"/>
+      <c r="A33" s="4" t="inlineStr"/>
+      <c r="B33" s="4" t="inlineStr"/>
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr"/>
       <c r="F33" s="6" t="inlineStr">
         <is>
           <t>[AOP-MEMORY]
@@ -1075,15 +1075,15 @@
 Área: Memory (v1.2)</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr"/>
-      <c r="H33" s="5" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr"/>
-      <c r="C34" s="5" t="inlineStr"/>
-      <c r="D34" s="5" t="inlineStr"/>
-      <c r="E34" s="5" t="inlineStr"/>
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr"/>
       <c r="F34" s="6" t="inlineStr">
         <is>
           <t>[AOP-API-SURFACES]
@@ -1091,8 +1091,232 @@
 Área: Platform API (v1.2)</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr"/>
-      <c r="H34" s="5" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr"/>
+      <c r="H34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-ORG-FOUNDATION]
+Virtual Organization Foundation
+Área: Virtual Organization (v1.2)</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="4" t="inlineStr"/>
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-ORG-BUDGET]
+Team Resource Governance &amp; Budget Control
+Área: Virtual Organization (v1.2)</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr"/>
+      <c r="B37" s="4" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-ORG-COORDINATION]
+Organizational Agent Coordination Foundation
+Área: Virtual Organization (v1.3)</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr"/>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-AGENT-CAPABILITY-GOVERNANCE]
+Agent Capability &amp; Responsibility Governance
+Área: Virtual Organization (v1.3)</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr"/>
+      <c r="H38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr"/>
+      <c r="B39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr"/>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-WORKFLOW-ORCHESTRATION]
+Workflow Orchestration &amp; Governed Task Assignment
+Área: Virtual Organization (v1.3)</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr"/>
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-WORKFLOW-VERIFICATION]
+Workflow Verification &amp; Result Validation
+Área: Workflow Governance (v1.3)</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr"/>
+      <c r="H40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr"/>
+      <c r="B41" s="4" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr"/>
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-HUMAN-OVERSIGHT]
+Human Oversight, Approval &amp; Escalation Governance
+Área: Workflow Governance (v1.3)</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-AGENT-LIFECYCLE-EVALUATION]
+Agent Lifecycle, Evaluation &amp; Governance
+Área: Virtual Organization (v1.3)</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr"/>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-AI-SOLUTIONS-FACTORY]
+AI Solutions Factory &amp; Blueprint Governance
+Área: Application Factory (v1.3)</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-ENTERPRISE-OPERATING-SYSTEM]
+AI Enterprise Operating System &amp; Executive Governance
+Área: Enterprise Strategy (v1.3)</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr"/>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-EXECUTIVE-ORCHESTRATOR]
+Executive Orchestrator &amp; Closed-Loop Business Operations
+Área: Executive Orchestration (v1.3)</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr"/>
+      <c r="B46" s="4" t="inlineStr"/>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-AUTONOMOUS-OPERATIONS-RUNTIME]
+Autonomous Operations Runtime &amp; Continuous Business Governance
+Área: Autonomous Operations (v1.3)</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-AUTONOMOUS-OPS-UI]
+Autonomous Operations Web Control Plane &amp; Front-End Governance
+Área: Web UI &amp; Control Plane (v1.3)</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr"/>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>[AOP-STREAMING]
+Reactive Operational Streaming (SSE)
+Área: Observability (v1.3)</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr"/>
+      <c r="H48" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3473,19 +3697,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
@@ -5898,82 +6122,1160 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
+          <t>AOP-ORG-FOUNDATION</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Virtual Organization Foundation</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Virtual Organization</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>Jerarquía multinivel de Organizaciones, Áreas, Equipos y Membresía gobernada de agentes con roles.</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>AOP-PROD-001</t>
+        </is>
+      </c>
+      <c r="I35" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/organization/</t>
+        </is>
+      </c>
+      <c r="J35" s="9" t="inlineStr">
+        <is>
+          <t>34 tests</t>
+        </is>
+      </c>
+      <c r="K35" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0027-virtual-organization-foundation.md</t>
+        </is>
+      </c>
+      <c r="L35" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 102</t>
+        </is>
+      </c>
+      <c r="M35" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N35" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O35" s="9" t="inlineStr">
+        <is>
+          <t>Jerarquía virtual</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>AOP-ORG-BUDGET</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Team Resource Governance &amp; Budget Control</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Virtual Organization</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Presupuestos y cuotas operacionales por equipo con control de concurrencia atómico (OCC).</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>v1.2</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>AOP-ORG-FOUNDATION</t>
+        </is>
+      </c>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/organization/team-resource-budget.ts</t>
+        </is>
+      </c>
+      <c r="J36" s="9" t="inlineStr">
+        <is>
+          <t>24 tests</t>
+        </is>
+      </c>
+      <c r="K36" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0028-team-resource-budget-governance.md</t>
+        </is>
+      </c>
+      <c r="L36" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 103</t>
+        </is>
+      </c>
+      <c r="M36" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N36" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O36" s="9" t="inlineStr">
+        <is>
+          <t>Fail-closed quotas</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>AOP-ORG-COORDINATION</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Organizational Agent Coordination Foundation</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Virtual Organization</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>Coordinación organizacional entre agentes, detección de ciclos, límites de profundidad y presupuestos.</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>AOP-ORG-BUDGET</t>
+        </is>
+      </c>
+      <c r="I37" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/organization/organizational-coordination.ts</t>
+        </is>
+      </c>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>23 tests</t>
+        </is>
+      </c>
+      <c r="K37" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0030-organizational-coordination-foundation.md</t>
+        </is>
+      </c>
+      <c r="L37" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 109</t>
+        </is>
+      </c>
+      <c r="M37" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N37" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O37" s="9" t="inlineStr">
+        <is>
+          <t>Multi-agent tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>AOP-AGENT-CAPABILITY-GOVERNANCE</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Agent Capability &amp; Responsibility Governance</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Virtual Organization</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Gobernanza formal de roles, responsabilidades, ciclo de vida de capacidades y descubrimiento.</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>AOP-ORG-COORDINATION</t>
+        </is>
+      </c>
+      <c r="I38" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/organization/agent-profile.ts</t>
+        </is>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>27 tests</t>
+        </is>
+      </c>
+      <c r="K38" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0031-agent-role-responsibility-capability-governance.md</t>
+        </is>
+      </c>
+      <c r="L38" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 110</t>
+        </is>
+      </c>
+      <c r="M38" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N38" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O38" s="9" t="inlineStr">
+        <is>
+          <t>Capacidades tipadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>AOP-WORKFLOW-ORCHESTRATION</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Workflow Orchestration &amp; Governed Task Assignment</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Virtual Organization</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>Orquestación de flujos de trabajo en DAG, asignación gobernada mediante PolicyGateway y cuotas.</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>AOP-AGENT-CAPABILITY-GOVERNANCE</t>
+        </is>
+      </c>
+      <c r="I39" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/workflow/</t>
+        </is>
+      </c>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>29 tests</t>
+        </is>
+      </c>
+      <c r="K39" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0032-workflow-orchestration-governed-task-assignment.md</t>
+        </is>
+      </c>
+      <c r="L39" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 111</t>
+        </is>
+      </c>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N39" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O39" s="9" t="inlineStr">
+        <is>
+          <t>DAG acíclico</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>AOP-WORKFLOW-VERIFICATION</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Workflow Verification &amp; Result Validation</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Workflow Governance</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Capa de verificación determinista con reglas/esquemas y segregación de funciones (SoD).</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>AOP-WORKFLOW-ORCHESTRATION</t>
+        </is>
+      </c>
+      <c r="I40" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/workflow/verification-result.ts</t>
+        </is>
+      </c>
+      <c r="J40" s="9" t="inlineStr">
+        <is>
+          <t>28 tests</t>
+        </is>
+      </c>
+      <c r="K40" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0033-workflow-verification-and-result-validation.md</t>
+        </is>
+      </c>
+      <c r="L40" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 112</t>
+        </is>
+      </c>
+      <c r="M40" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N40" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O40" s="9" t="inlineStr">
+        <is>
+          <t>Segregación SoD</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>AOP-HUMAN-OVERSIGHT</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Human Oversight, Approval &amp; Escalation Governance</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Workflow Governance</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Supervisión humana, aprobación y escalamiento gobernado con prevención de bypass y OCC.</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>AOP-WORKFLOW-VERIFICATION</t>
+        </is>
+      </c>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/workflow/oversight-request.ts</t>
+        </is>
+      </c>
+      <c r="J41" s="9" t="inlineStr">
+        <is>
+          <t>26 tests</t>
+        </is>
+      </c>
+      <c r="K41" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0034-human-oversight-approval-and-escalation-governance.md</t>
+        </is>
+      </c>
+      <c r="L41" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 113</t>
+        </is>
+      </c>
+      <c r="M41" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N41" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O41" s="9" t="inlineStr">
+        <is>
+          <t>Control humano</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>AOP-AGENT-LIFECYCLE-EVALUATION</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle, Evaluation &amp; Governance</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Virtual Organization</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Ciclo de vida de agentes, evaluaciones cuantitativas deterministas y elegibilidad estricta.</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>AOP-HUMAN-OVERSIGHT</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/agent/agent-profile.ts</t>
+        </is>
+      </c>
+      <c r="J42" s="9" t="inlineStr">
+        <is>
+          <t>28 tests</t>
+        </is>
+      </c>
+      <c r="K42" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0035-agent-lifecycle-evaluation-and-governance.md</t>
+        </is>
+      </c>
+      <c r="L42" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 114</t>
+        </is>
+      </c>
+      <c r="M42" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N42" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O42" s="9" t="inlineStr">
+        <is>
+          <t>Métricas cuantitativas</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>AOP-AI-SOLUTIONS-FACTORY</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>AI Solutions Factory &amp; Blueprint Governance</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Application Factory</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Fábrica de soluciones de IA, planos arquitectónicos declarativos y ciclo de vida de soluciones.</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>AOP-AGENT-LIFECYCLE-EVALUATION</t>
+        </is>
+      </c>
+      <c r="I43" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/solution/</t>
+        </is>
+      </c>
+      <c r="J43" s="9" t="inlineStr">
+        <is>
+          <t>32 tests</t>
+        </is>
+      </c>
+      <c r="K43" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0036-ai-solutions-factory-and-blueprint-governance.md</t>
+        </is>
+      </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 115</t>
+        </is>
+      </c>
+      <c r="M43" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N43" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O43" s="9" t="inlineStr">
+        <is>
+          <t>Planos declarativos</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>AOP-ENTERPRISE-OPERATING-SYSTEM</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>AI Enterprise Operating System &amp; Executive Governance</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Enterprise Strategy</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Sistema operativo empresarial impulsado por IA y cadena de valor estratégica.</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
+        <is>
+          <t>AOP-AI-SOLUTIONS-FACTORY</t>
+        </is>
+      </c>
+      <c r="I44" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/business/</t>
+        </is>
+      </c>
+      <c r="J44" s="9" t="inlineStr">
+        <is>
+          <t>26 tests</t>
+        </is>
+      </c>
+      <c r="K44" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0037-ai-enterprise-operating-system-and-executive-governance.md</t>
+        </is>
+      </c>
+      <c r="L44" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 116</t>
+        </is>
+      </c>
+      <c r="M44" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N44" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O44" s="9" t="inlineStr">
+        <is>
+          <t>Estrategia ejecutiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>AOP-EXECUTIVE-ORCHESTRATOR</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Executive Orchestrator &amp; Closed-Loop Business Operations</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Executive Orchestration</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Orquestación ejecutiva de bucle cerrado, instantáneas inmutables y re-planificación acotada.</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>AOP-ENTERPRISE-OPERATING-SYSTEM</t>
+        </is>
+      </c>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/executive/</t>
+        </is>
+      </c>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>28 tests</t>
+        </is>
+      </c>
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0038-executive-orchestrator-and-closed-loop-business-operations.md</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 117</t>
+        </is>
+      </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N45" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O45" s="9" t="inlineStr">
+        <is>
+          <t>Bucle cerrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>AOP-AUTONOMOUS-OPERATIONS-RUNTIME</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Autonomous Operations Runtime &amp; Continuous Business Governance</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Autonomous Operations</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Daemon 24/7 de operaciones autónomas continuas, leases concurrentes y circuit breaker.</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>AOP-EXECUTIVE-ORCHESTRATOR</t>
+        </is>
+      </c>
+      <c r="I46" s="9" t="inlineStr">
+        <is>
+          <t>src/domain/autonomous/</t>
+        </is>
+      </c>
+      <c r="J46" s="9" t="inlineStr">
+        <is>
+          <t>16 tests</t>
+        </is>
+      </c>
+      <c r="K46" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0039-autonomous-operations-runtime-and-continuous-business-governance.md</t>
+        </is>
+      </c>
+      <c r="L46" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 118</t>
+        </is>
+      </c>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N46" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O46" s="9" t="inlineStr">
+        <is>
+          <t>Daemon operacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>AOP-AUTONOMOUS-OPS-UI</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Autonomous Operations Web Control Plane &amp; Front-End Governance</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Web UI &amp; Control Plane</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Consola operativa #tab-operations, tabla de triggers, cadena de 6 fases y 0 innerHTML.</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>AOP-AUTONOMOUS-OPERATIONS-RUNTIME</t>
+        </is>
+      </c>
+      <c r="I47" s="9" t="inlineStr">
+        <is>
+          <t>src/platform/web/app.js</t>
+        </is>
+      </c>
+      <c r="J47" s="9" t="inlineStr">
+        <is>
+          <t>14 tests</t>
+        </is>
+      </c>
+      <c r="K47" s="9" t="inlineStr">
+        <is>
+          <t>docs/AUTONOMOUS_OPERATIONS.md</t>
+        </is>
+      </c>
+      <c r="L47" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 101</t>
+        </is>
+      </c>
+      <c r="M47" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N47" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O47" s="9" t="inlineStr">
+        <is>
+          <t>Control plane web</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>AOP-STREAMING</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Reactive Operational Streaming (SSE)</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>Streaming reactivo de eventos operacionales vía Server-Sent Events y replay.</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>AOP-PROD-001</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>src/application/observability/event-stream-adapter.ts</t>
+        </is>
+      </c>
+      <c r="J48" s="9" t="inlineStr">
+        <is>
+          <t>8 tests</t>
+        </is>
+      </c>
+      <c r="K48" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0029-reactive-operational-streaming-sse.md</t>
+        </is>
+      </c>
+      <c r="L48" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 108</t>
+        </is>
+      </c>
+      <c r="M48" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N48" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O48" s="9" t="inlineStr">
+        <is>
+          <t>SSE streaming</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
           <t>AOP-V1-EXIT</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>Certificación Final de Criterios de Producción</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C49" s="9" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Auditoría y ejecución de pruebas de carga para cumplimiento de criterios de release formal.</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>BACKLOG</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Auditoría y certificación integral de criterios de release formal para producción masiva.</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>VALIDATION</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr">
-        <is>
-          <t>v1.2</t>
-        </is>
-      </c>
-      <c r="H35" s="9" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
         <is>
           <t>Todos los anteriores</t>
         </is>
       </c>
-      <c r="I35" s="9" t="inlineStr">
+      <c r="I49" s="9" t="inlineStr">
+        <is>
+          <t>docs/RELEASE_CERTIFICATION_V1.md</t>
+        </is>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>1354 tests</t>
+        </is>
+      </c>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>docs/V1_EXIT_CRITERIA.md</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 106</t>
+        </is>
+      </c>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N49" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J35" s="9" t="inlineStr">
-        <is>
-          <t>0 tests</t>
-        </is>
-      </c>
-      <c r="K35" s="9" t="inlineStr">
-        <is>
-          <t>docs/V1_EXIT_CRITERIA.md</t>
-        </is>
-      </c>
-      <c r="L35" s="9" t="inlineStr">
-        <is>
-          <t>Prompt 101+</t>
-        </is>
-      </c>
-      <c r="M35" s="9" t="inlineStr">
-        <is>
-          <t>Platform Core</t>
-        </is>
-      </c>
-      <c r="N35" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="O35" s="9" t="inlineStr">
+      <c r="O49" s="9" t="inlineStr">
         <is>
           <t>Criterios formales</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O35"/>
+  <autoFilter ref="A4:O49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(phase-71): enterprise authentication, api authorization and credential governance
</commit_message>
<xml_diff>
--- a/AI_Operating_Platform_Roadmap.xlsx
+++ b/AI_Operating_Platform_Roadmap.xlsx
@@ -23,7 +23,7 @@
     <sheet name="14_DASHBOARD" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_MASTER_ROADMAP'!$A$4:$O$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_MASTER_ROADMAP'!$A$4:$O$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1038,7 +1038,7 @@
       <c r="E31" s="4" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>[AOP-AUTH]
+          <t>[AOP-AUTH-JWT]
 Proveedor de Autenticación OIDC / JWT Producción
 Área: Security (v1.2)</t>
         </is>
@@ -1310,13 +1310,29 @@
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="6" t="inlineStr">
         <is>
+          <t>[AOP-AUTH]
+Enterprise Authentication, API Authorization &amp; Credential Governance
+Área: Security (v1.3)</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr"/>
+      <c r="H48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr"/>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
           <t>[AOP-STREAMING]
 Reactive Operational Streaming (SSE)
 Área: Observability (v1.3)</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr"/>
+      <c r="H49" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3306,7 +3322,7 @@
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>1.1.0</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -3323,7 +3339,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>985 PASS (0 FAIL)</t>
+          <t>1391 PASS (0 FAIL)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -3340,7 +3356,7 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>11 Suites</t>
+          <t>59 Suites</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -3357,7 +3373,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>31 Iniciativas</t>
+          <t>46 Iniciativas</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -3374,7 +3390,7 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>30 Iniciativas (96.8%)</t>
+          <t>45 Iniciativas (97.8%)</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -3386,12 +3402,12 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Iniciativas en Backlog Formal (BACKLOG)</t>
+          <t>Iniciativas en Validación (VALIDATION)</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>1 Iniciativa (3.2%)</t>
+          <t>1 Iniciativa (2.2%)</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -3459,12 +3475,12 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>36 ADRs Catalogados</t>
+          <t>50 ADRs Catalogados</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>docs/decisions/ (ADR 0001 al 0026 + Serie ADR-001..010)</t>
+          <t>docs/decisions/ (ADR 0001 al 0040 + Serie ADR-001..010)</t>
         </is>
       </c>
     </row>
@@ -3697,7 +3713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5814,7 +5830,7 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>AOP-AUTH</t>
+          <t>AOP-AUTH-JWT</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -7123,22 +7139,22 @@
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>AOP-STREAMING</t>
+          <t>AOP-AUTH</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Reactive Operational Streaming (SSE)</t>
+          <t>Enterprise Authentication, API Authorization &amp; Credential Governance</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Observability</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Streaming reactivo de eventos operacionales vía Server-Sent Events y replay.</t>
+          <t>Gobernanza de credenciales API empresariales (zero-plaintext SHA-256), vinculación de Principal, scopes, reconciliación y rotación.</t>
         </is>
       </c>
       <c r="E48" s="10" t="inlineStr">
@@ -7148,7 +7164,7 @@
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="G48" s="11" t="inlineStr">
@@ -7158,27 +7174,27 @@
       </c>
       <c r="H48" s="9" t="inlineStr">
         <is>
-          <t>AOP-PROD-001</t>
+          <t>AOP-AUTONOMOUS-OPS-UI</t>
         </is>
       </c>
       <c r="I48" s="9" t="inlineStr">
         <is>
-          <t>src/application/observability/event-stream-adapter.ts</t>
+          <t>src/domain/security/api-credential.ts</t>
         </is>
       </c>
       <c r="J48" s="9" t="inlineStr">
         <is>
-          <t>8 tests</t>
+          <t>37 tests</t>
         </is>
       </c>
       <c r="K48" s="9" t="inlineStr">
         <is>
-          <t>docs/decisions/0029-reactive-operational-streaming-sse.md</t>
+          <t>docs/decisions/0040-enterprise-api-authentication-and-credential-governance.md</t>
         </is>
       </c>
       <c r="L48" s="9" t="inlineStr">
         <is>
-          <t>Prompt 108</t>
+          <t>Prompt 102</t>
         </is>
       </c>
       <c r="M48" s="9" t="inlineStr">
@@ -7193,89 +7209,166 @@
       </c>
       <c r="O48" s="9" t="inlineStr">
         <is>
-          <t>SSE streaming</t>
+          <t>Zero-plaintext &amp; Scopes</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
+          <t>AOP-STREAMING</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Reactive Operational Streaming (SSE)</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Streaming reactivo de eventos operacionales vía Server-Sent Events y replay.</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>AOP-PROD-001</t>
+        </is>
+      </c>
+      <c r="I49" s="9" t="inlineStr">
+        <is>
+          <t>src/application/observability/event-stream-adapter.ts</t>
+        </is>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>8 tests</t>
+        </is>
+      </c>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>docs/decisions/0029-reactive-operational-streaming-sse.md</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>Prompt 108</t>
+        </is>
+      </c>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>Platform Core</t>
+        </is>
+      </c>
+      <c r="N49" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O49" s="9" t="inlineStr">
+        <is>
+          <t>SSE streaming</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
           <t>AOP-V1-EXIT</t>
         </is>
       </c>
-      <c r="B49" s="9" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>Certificación Final de Criterios de Producción</t>
         </is>
       </c>
-      <c r="C49" s="9" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>Governance</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr">
+      <c r="D50" s="9" t="inlineStr">
         <is>
           <t>Auditoría y certificación integral de criterios de release formal para producción masiva.</t>
         </is>
       </c>
-      <c r="E49" s="12" t="inlineStr">
+      <c r="E50" s="12" t="inlineStr">
         <is>
           <t>VALIDATION</t>
         </is>
       </c>
-      <c r="F49" s="11" t="inlineStr">
+      <c r="F50" s="11" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr">
+      <c r="G50" s="11" t="inlineStr">
         <is>
           <t>v1.3</t>
         </is>
       </c>
-      <c r="H49" s="9" t="inlineStr">
+      <c r="H50" s="9" t="inlineStr">
         <is>
           <t>Todos los anteriores</t>
         </is>
       </c>
-      <c r="I49" s="9" t="inlineStr">
+      <c r="I50" s="9" t="inlineStr">
         <is>
           <t>docs/RELEASE_CERTIFICATION_V1.md</t>
         </is>
       </c>
-      <c r="J49" s="9" t="inlineStr">
-        <is>
-          <t>1354 tests</t>
-        </is>
-      </c>
-      <c r="K49" s="9" t="inlineStr">
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>1391 tests</t>
+        </is>
+      </c>
+      <c r="K50" s="9" t="inlineStr">
         <is>
           <t>docs/V1_EXIT_CRITERIA.md</t>
         </is>
       </c>
-      <c r="L49" s="9" t="inlineStr">
+      <c r="L50" s="9" t="inlineStr">
         <is>
           <t>Prompt 106</t>
         </is>
       </c>
-      <c r="M49" s="9" t="inlineStr">
+      <c r="M50" s="9" t="inlineStr">
         <is>
           <t>Platform Core</t>
         </is>
       </c>
-      <c r="N49" s="9" t="inlineStr">
+      <c r="N50" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O49" s="9" t="inlineStr">
+      <c r="O50" s="9" t="inlineStr">
         <is>
           <t>Criterios formales</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O49"/>
+  <autoFilter ref="A4:O50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8394,7 +8487,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>AOP-AUTH</t>
+          <t>AOP-AUTH-JWT</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">

</xml_diff>